<commit_message>
자동 업데이트: data.xlsx (2026-04-28 23:31:47)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2195293818081/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2212454164649/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="13_ncr:1_{27431DA6-BDD5-40A6-9189-C5D7C0B6EDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11ABF5F9-5E15-4545-9BF4-4A23A7E61593}"/>
+  <xr:revisionPtr revIDLastSave="123" documentId="13_ncr:1_{27431DA6-BDD5-40A6-9189-C5D7C0B6EDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61022FF7-F32F-4B52-80BE-2A8F3207EB3A}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta" sheetId="1" r:id="rId1"/>
@@ -1741,7 +1741,9 @@
       <c r="B12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="2">
+        <v>5.1000000000000004E-3</v>
+      </c>
       <c r="D12" s="2">
         <v>1.3999999999999999E-2</v>
       </c>

</xml_diff>

<commit_message>
자동 업데이트: data.xlsx (2026-05-11 11:31:01)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2212454164649/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2195293818081/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="13_ncr:1_{27431DA6-BDD5-40A6-9189-C5D7C0B6EDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61022FF7-F32F-4B52-80BE-2A8F3207EB3A}"/>
+  <xr:revisionPtr revIDLastSave="151" documentId="13_ncr:1_{27431DA6-BDD5-40A6-9189-C5D7C0B6EDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD160BED-F065-49B0-BADE-EC486764A14F}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="189">
   <si>
     <t>Key</t>
   </si>
@@ -828,6 +828,17 @@
   </si>
   <si>
     <t>▶ ASRS Shuttle PM(#49~64) 완료, ASRS Rack PM(5,6F) 완료</t>
+  </si>
+  <si>
+    <t>2026.Apr</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>▶ ASRS Shuttle PM(#65~80) 완료, ASRS Rack PM(3,4F) 완료</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>▶ Conveyor check-up by Millbang Korea 완료 (4/26~4/28)</t>
   </si>
 </sst>
 </file>
@@ -1742,7 +1753,7 @@
         <v>17</v>
       </c>
       <c r="C12" s="2">
-        <v>5.1000000000000004E-3</v>
+        <v>9.7999999999999997E-3</v>
       </c>
       <c r="D12" s="2">
         <v>1.3999999999999999E-2</v>
@@ -1907,7 +1918,9 @@
       <c r="B24" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="2">
+        <v>1E-3</v>
+      </c>
       <c r="D24" s="2">
         <v>6.0000000000000001E-3</v>
       </c>
@@ -2071,7 +2084,9 @@
       <c r="B36" t="s">
         <v>16</v>
       </c>
-      <c r="C36" s="2"/>
+      <c r="C36" s="2">
+        <v>6.0000000000000001E-3</v>
+      </c>
       <c r="D36" s="2">
         <v>2.5000000000000001E-2</v>
       </c>
@@ -2268,6 +2283,9 @@
       <c r="B12" t="s">
         <v>17</v>
       </c>
+      <c r="C12">
+        <v>0.08</v>
+      </c>
       <c r="D12">
         <v>0.25</v>
       </c>
@@ -2430,6 +2448,9 @@
       <c r="B24" t="s">
         <v>15</v>
       </c>
+      <c r="C24">
+        <v>0.21</v>
+      </c>
       <c r="D24">
         <v>0.3</v>
       </c>
@@ -2591,6 +2612,9 @@
       </c>
       <c r="B36" t="s">
         <v>16</v>
+      </c>
+      <c r="C36">
+        <v>0.06</v>
       </c>
       <c r="D36">
         <v>7.0000000000000007E-2</v>
@@ -4190,7 +4214,9 @@
       <c r="C112" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D112" s="14"/>
+      <c r="D112" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="113" spans="1:4" hidden="1">
       <c r="A113" s="6" t="s">
@@ -4202,7 +4228,9 @@
       <c r="C113" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D113" s="14"/>
+      <c r="D113" s="14">
+        <v>8.9999999999999998E-4</v>
+      </c>
     </row>
     <row r="114" spans="1:4" hidden="1">
       <c r="A114" s="6" t="s">
@@ -4214,7 +4242,9 @@
       <c r="C114" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D114" s="14"/>
+      <c r="D114" s="14">
+        <v>1E-4</v>
+      </c>
     </row>
     <row r="115" spans="1:4" hidden="1">
       <c r="A115" s="6" t="s">
@@ -4226,7 +4256,9 @@
       <c r="C115" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D115" s="14"/>
+      <c r="D115" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="116" spans="1:4" hidden="1">
       <c r="A116" s="6" t="s">
@@ -4238,7 +4270,9 @@
       <c r="C116" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D116" s="14"/>
+      <c r="D116" s="14">
+        <v>4.0000000000000002E-4</v>
+      </c>
     </row>
     <row r="117" spans="1:4" hidden="1">
       <c r="A117" s="6" t="s">
@@ -4250,7 +4284,9 @@
       <c r="C117" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D117" s="14"/>
+      <c r="D117" s="14">
+        <v>4.0000000000000002E-4</v>
+      </c>
     </row>
     <row r="118" spans="1:4" ht="16.5" hidden="1" customHeight="1">
       <c r="A118" s="6" t="s">
@@ -4262,7 +4298,9 @@
       <c r="C118" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D118" s="14"/>
+      <c r="D118" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="119" spans="1:4" ht="16.5" hidden="1" customHeight="1">
       <c r="A119" s="6" t="s">
@@ -4274,7 +4312,9 @@
       <c r="C119" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D119" s="14"/>
+      <c r="D119" s="14">
+        <v>5.1000000000000004E-3</v>
+      </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="6" t="s">
@@ -4286,7 +4326,9 @@
       <c r="C120" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D120" s="14"/>
+      <c r="D120" s="14">
+        <v>1.4E-3</v>
+      </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="6" t="s">
@@ -4298,7 +4340,9 @@
       <c r="C121" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D121" s="14"/>
+      <c r="D121" s="14">
+        <v>6.1000000000000004E-3</v>
+      </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="6" t="s">
@@ -4310,7 +4354,9 @@
       <c r="C122" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D122" s="14"/>
+      <c r="D122" s="14">
+        <v>2.3E-3</v>
+      </c>
     </row>
     <row r="123" spans="1:4" hidden="1">
       <c r="A123" s="6" t="s">
@@ -4951,19 +4997,31 @@
       <c r="G24" s="6"/>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="13"/>
-      <c r="B25" s="6"/>
+      <c r="A25" s="12">
+        <v>46113</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>62</v>
+      </c>
       <c r="C25" s="6"/>
-      <c r="D25" s="7"/>
+      <c r="D25" s="7" t="s">
+        <v>177</v>
+      </c>
       <c r="E25" s="7"/>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="13"/>
-      <c r="B26" s="6"/>
+      <c r="A26" s="12">
+        <v>46113</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>17</v>
+      </c>
       <c r="C26" s="6"/>
-      <c r="D26" s="7"/>
+      <c r="D26" s="7" t="s">
+        <v>177</v>
+      </c>
       <c r="E26" s="7"/>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
@@ -5634,12 +5692,20 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="6"/>
-      <c r="B27" s="6"/>
+      <c r="A27" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="6"/>
-      <c r="B28" s="6"/>
+      <c r="A28" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="6"/>

</xml_diff>

<commit_message>
자동 업데이트: data.xlsx (2026-05-12 13:01:17)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2195293818081/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2225533485465/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="151" documentId="13_ncr:1_{27431DA6-BDD5-40A6-9189-C5D7C0B6EDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD160BED-F065-49B0-BADE-EC486764A14F}"/>
+  <xr:revisionPtr revIDLastSave="152" documentId="13_ncr:1_{27431DA6-BDD5-40A6-9189-C5D7C0B6EDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D0C3B8B-27F8-42B7-AB7F-F114721AC594}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="189">
   <si>
     <t>Key</t>
   </si>
@@ -5018,7 +5018,9 @@
       <c r="B26" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="6"/>
+      <c r="C26" s="9" t="s">
+        <v>32</v>
+      </c>
       <c r="D26" s="7" t="s">
         <v>177</v>
       </c>

</xml_diff>

<commit_message>
자동 업데이트: data.xlsx (2026-05-12 13:08:39)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2225533485465/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="152" documentId="13_ncr:1_{27431DA6-BDD5-40A6-9189-C5D7C0B6EDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D0C3B8B-27F8-42B7-AB7F-F114721AC594}"/>
+  <xr:revisionPtr revIDLastSave="156" documentId="13_ncr:1_{27431DA6-BDD5-40A6-9189-C5D7C0B6EDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{699022FB-406E-495E-879B-6CDAB49D9803}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="192">
   <si>
     <t>Key</t>
   </si>
@@ -839,6 +839,15 @@
   </si>
   <si>
     <t>▶ Conveyor check-up by Millbang Korea 완료 (4/26~4/28)</t>
+  </si>
+  <si>
+    <t>TK02.01.017KU Motorized roller 고장</t>
+  </si>
+  <si>
+    <t>1hr15min</t>
+  </si>
+  <si>
+    <t>Mezzanine 2F TK02.01.017KU 구간 Roller 동작 안됨</t>
   </si>
 </sst>
 </file>
@@ -5011,7 +5020,7 @@
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" ht="30">
       <c r="A26" s="12">
         <v>46113</v>
       </c>
@@ -5022,10 +5031,14 @@
         <v>32</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E26" s="7"/>
-      <c r="F26" s="6"/>
+        <v>191</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>190</v>
+      </c>
       <c r="G26" s="6"/>
     </row>
     <row r="27" spans="1:7">

</xml_diff>